<commit_message>
📊 Excel更新: Carbon+Three.js+Remotion全→✅ 链接到位
</commit_message>
<xml_diff>
--- a/skillu-tools.xlsx
+++ b/skillu-tools.xlsx
@@ -1139,14 +1139,14 @@
           <t>npx carbon-now code.py</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>⚠️</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>📄 调用规范</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
@@ -1239,14 +1239,14 @@
           <t>JS→3D场景</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>⚠️</t>
-        </is>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>📄 调用规范</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
@@ -1289,14 +1289,14 @@
           <t>React→MP4视频</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>⚠️</t>
-        </is>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>📄 调用规范</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
@@ -2080,40 +2080,43 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId59"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🔄 Trufflehog→Gitleaks(秒抓密钥) Firecrawl→Jina Reader(零配置替代)
</commit_message>
<xml_diff>
--- a/skillu-tools.xlsx
+++ b/skillu-tools.xlsx
@@ -1511,7 +1511,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Trufflehog</t>
+          <t>Gitleaks</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1526,22 +1526,22 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>3.95.5</t>
+          <t>8.30.1</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>brew install trufflehog</t>
+          <t>brew install gitleaks</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>trufflehog git file://.</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>⚠️</t>
+          <t>gitleaks detect --source .</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
@@ -1991,12 +1991,12 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>⚠️</t>
-        </is>
-      </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>→Jina</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>Jina代替</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
@@ -2114,9 +2114,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>